<commit_message>
Auto update Pengadaan 2026-10-26 10:14:50
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
@@ -819,19 +819,19 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>986719971</v>
+        <v>985113021</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>708189164</v>
+        <v>706582214</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>282732900</v>
@@ -1583,22 +1583,22 @@
         <v>283301771</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>50379150</v>
+        <v>65316100</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>46526860</v>
+        <v>61364960</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>232922621</v>
+        <v>217985671</v>
       </c>
     </row>
     <row r="32" ht="45" customHeight="1">
@@ -2227,22 +2227,22 @@
         <v>606936476</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>274236748</v>
+        <v>278141173</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>250171300</v>
+        <v>253688800</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J49" s="10" t="n">
-        <v>332699728</v>
+        <v>328795303</v>
       </c>
     </row>
     <row r="50" ht="45" customHeight="1">
@@ -3347,28 +3347,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4005</v>
+        <v>4004</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>34829718047</v>
+        <v>34828111097</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>7742395237</v>
+        <v>7759629662</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6904072474.6</v>
+        <v>6922428074.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3474</v>
+        <v>3468</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27087322810</v>
+        <v>27068481435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-26 12:09:41
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
@@ -924,13 +924,13 @@
         <v>122</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>756952316</v>
+        <v>756952315</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F15" s="10" t="n">
-        <v>63250745</v>
+        <v>63250744</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>2</v>
@@ -1004,35 +1004,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1154,35 +1146,27 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G20" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>3839600910</v>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
@@ -1308,13 +1292,13 @@
         <v>93</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1145584728</v>
+        <v>1148350728</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>55769294</v>
+        <v>58535294</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>6</v>
@@ -1339,22 +1323,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>414639535</v>
+        <v>403884747</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>84907554</v>
+        <v>74152766</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>78869208</v>
+        <v>128214258</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>62</v>
@@ -1373,22 +1357,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>963345953</v>
+        <v>961842399</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>137583844</v>
+        <v>136080290</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>116218702</v>
+        <v>1520271914</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>109</v>
@@ -1407,22 +1391,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>497942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>338050900</v>
+        <v>3037348900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1478,13 +1462,13 @@
         <v>100</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>900575817</v>
+        <v>890948817</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>38508000</v>
+        <v>28881000</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>1</v>
@@ -1512,13 +1496,13 @@
         <v>187</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>2559551299</v>
+        <v>2550047146</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>58</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>1228508400</v>
+        <v>1219004247</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>58</v>
@@ -1543,22 +1527,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>90550292</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>86612607</v>
+        <v>236612607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>44</v>
@@ -1580,13 +1564,13 @@
         <v>52</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>283301771</v>
+        <v>283157746</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>14</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>65316100</v>
+        <v>65172075</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>14</v>
@@ -1614,13 +1598,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>767894130</v>
+        <v>764274671</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1648,13 +1632,13 @@
         <v>44</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>366634933</v>
+        <v>278301799</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>108974684</v>
+        <v>20641550</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1716,13 +1700,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>463972148</v>
+        <v>463836830</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1750,13 +1734,13 @@
         <v>76</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>761771973</v>
+        <v>761250273</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>13</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>334343818</v>
+        <v>333822118</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>13</v>
@@ -1781,28 +1765,28 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>1092264791</v>
+        <v>854862891</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>412496502</v>
+        <v>224284602</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>402113040</v>
+        <v>1186117670</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>679768289</v>
+        <v>630578289</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -1818,13 +1802,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>384332451</v>
+        <v>382731831</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>12</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>101993338</v>
+        <v>100392718</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>12</v>
@@ -1849,22 +1833,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>1262512215</v>
+        <v>1236982215</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>391109425</v>
+        <v>365579425</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>387344886</v>
+        <v>427421436</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>84</v>
@@ -1988,13 +1972,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>708077545</v>
+        <v>727698127</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2019,22 +2003,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>340998868</v>
+        <v>270482868</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>151137140</v>
+        <v>80621140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>18</v>
@@ -2103,22 +2087,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1100276809</v>
+        <v>1148929219</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>121983128</v>
+        <v>318350703</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>163</v>
@@ -2224,13 +2208,13 @@
         <v>99</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>606936476</v>
+        <v>605011476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>31</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>278141173</v>
+        <v>276216173</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>31</v>
@@ -2339,30 +2323,24 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E52" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G52" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>65401200</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3132,13 +3110,13 @@
         <v>41</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>330321582</v>
+        <v>323431257</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3163,22 +3141,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>158730000</v>
+        <v>2359971000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3284,7 +3262,7 @@
         <v>113</v>
       </c>
       <c r="D75" s="10" t="n">
-        <v>1433154546</v>
+        <v>1398754546</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3302,7 +3280,7 @@
         <v>95</v>
       </c>
       <c r="J75" s="10" t="n">
-        <v>1013280360</v>
+        <v>978880360</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3318,13 +3296,13 @@
         <v>145</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1492289470</v>
+        <v>1484655470</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>24</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>207985114</v>
+        <v>200351114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>24</v>
@@ -3347,28 +3325,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4004</v>
+        <v>4054</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>34828111097</v>
+        <v>34389109112</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>536</v>
+        <v>585</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>7759629662</v>
+        <v>7404217677</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>536</v>
+        <v>585</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6922428074.6</v>
+        <v>20159216179.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27068481435</v>
+        <v>26984891435</v>
       </c>
     </row>
   </sheetData>
@@ -3789,13 +3767,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4221,45 +4199,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4291,29 +4253,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>111200910</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>111200910</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -4536,34 +4514,50 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>323734637</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>54773006</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="K24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="9" t="n">
-        <v>49345050</v>
+        <v>268961631</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M24" s="7" t="n">
         <v>3</v>
@@ -4582,34 +4576,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>1848714675</v>
+        <v>1679001832</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>1225542538</v>
+        <v>1055829695</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>896262562</v>
+        <v>819807063</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>896262562</v>
+        <v>819807063</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>334523972</v>
+        <v>258068473</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>7</v>
@@ -4828,28 +4822,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
@@ -4881,13 +4875,13 @@
         <v>7</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>477133090</v>
+        <v>490395090</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>66310000</v>
+        <v>79572000</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
@@ -5081,13 +5075,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>1668288113</v>
+        <v>1667542131</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>886469138</v>
+        <v>885723156</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5131,13 +5125,13 @@
         <v>39</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>5044312982</v>
+        <v>5043896732</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>36</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>4775708657</v>
+        <v>4775292407</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>36</v>
@@ -5178,40 +5172,40 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>3308825552</v>
+        <v>2771677052</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>1839090451</v>
+        <v>1487941951</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1791219523</v>
+        <v>1444011523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1581713573</v>
+        <v>1234505573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L37" s="10" t="n">
-        <v>713727983</v>
+        <v>366519983</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N37" s="10" t="n">
-        <v>1469735101</v>
+        <v>1283735101</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -5286,28 +5280,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>4655680948</v>
+        <v>4402582653</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>2674384586</v>
+        <v>2421286291</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2613571243</v>
+        <v>2388524693</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2438894693</v>
+        <v>2253924693</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>1</v>
@@ -5560,28 +5554,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>547117650</v>
+        <v>475135300</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>2</v>
@@ -5676,28 +5670,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>932380105</v>
+        <v>716222170</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>448555830</v>
+        <v>252188255</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>309615830</v>
+        <v>113248255</v>
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
@@ -6020,34 +6014,38 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>559836352</v>
+        <v>319983894</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" s="9" t="n">
-        <v>301830114</v>
+        <v>61977656</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>68020787</v>
+        <v>2619587</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="K52" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="L52" s="9" t="n">
-        <v>65401200</v>
+        <v>2619587</v>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M52" s="7" t="n">
         <v>3</v>
@@ -7189,13 +7187,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>423288615</v>
+        <v>392285593</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7456,28 +7454,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>3401653729</v>
+        <v>3551653729</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>564698247</v>
+        <v>714698247</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -7504,40 +7502,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>901</v>
+        <v>885</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>106658823826</v>
+        <v>105168673685</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>66058453615</v>
+        <v>64754303474</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>528</v>
+        <v>513</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64159073617.41</v>
+        <v>63275727355.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>370</v>
+        <v>356</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>45929979518.03</v>
+        <v>45086709806.03</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1723429295</v>
+        <v>1185019546</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>40600370211</v>
+        <v>40414370211</v>
       </c>
     </row>
   </sheetData>
@@ -8347,28 +8345,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>26642121741</v>
+        <v>24845621741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>26642121741</v>
+        <v>24845621741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8454,29 +8452,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8508,29 +8522,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>1081900000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>1081900000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -8566,13 +8596,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8620,7 +8650,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
@@ -8666,7 +8696,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8799,40 +8829,40 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>49096492181</v>
+        <v>6460249182</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>47632716881</v>
+        <v>4916473882</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2829407037</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2829407037</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>2945468782</v>
+        <v>1712457037</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N25" s="10" t="n">
-        <v>1463775300</v>
+        <v>1543775300</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -9483,34 +9513,38 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>5765940896</v>
+        <v>4892340896</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2946694000</v>
+        <v>2073094000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>2509890630</v>
+        <v>2073094000</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>2509890630</v>
-      </c>
-      <c r="K37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="10" t="n">
-        <v>436796630</v>
+        <v>2073094000</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9599,28 +9633,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>3813601480</v>
+        <v>3962367980</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3013841480</v>
+        <v>3162607980</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>2</v>
@@ -9822,13 +9856,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11749,28 +11783,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>14398798637</v>
+        <v>7792798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -11961,28 +11995,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>7133067600</v>
+        <v>6783067600</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>3294207800</v>
+        <v>2944207800</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -12009,40 +12043,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>245</v>
+        <v>213</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>185102594591</v>
+        <v>131385975180</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147457910043</v>
+        <v>93666790632</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71036708305.01001</v>
+        <v>64029064462.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>67648469205</v>
+        <v>60640825362</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4430709261</v>
+        <v>2760900886</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>83</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>37644684548</v>
+        <v>37719184548</v>
       </c>
     </row>
   </sheetData>
@@ -13031,13 +13065,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13081,29 +13115,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>2646500000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>2646500000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -13486,28 +13536,40 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>5399320575</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>2699298000</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="9" t="n">
-        <v>2699298000</v>
+        <v>2699320575</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -16950,28 +17012,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>256072475553</v>
+        <v>250632775553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147115370800</v>
+        <v>141675670800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>